<commit_message>
Daily dashboard refresh 2026-01-20 02:49
</commit_message>
<xml_diff>
--- a/data/Fail.xlsx
+++ b/data/Fail.xlsx
@@ -2549,7 +2549,7 @@
         <v>609</v>
       </c>
       <c r="BE2" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="3" spans="1:57">
@@ -2701,7 +2701,7 @@
         <v>609</v>
       </c>
       <c r="BE3" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="4" spans="1:57">
@@ -2844,7 +2844,7 @@
         <v>609</v>
       </c>
       <c r="BE4" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="5" spans="1:57">
@@ -2993,7 +2993,7 @@
         <v>609</v>
       </c>
       <c r="BE5" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="6" spans="1:57">
@@ -3145,7 +3145,7 @@
         <v>609</v>
       </c>
       <c r="BE6" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="7" spans="1:57">
@@ -3297,7 +3297,7 @@
         <v>609</v>
       </c>
       <c r="BE7" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="8" spans="1:57">
@@ -3440,7 +3440,7 @@
         <v>609</v>
       </c>
       <c r="BE8" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="9" spans="1:57">
@@ -3592,7 +3592,7 @@
         <v>609</v>
       </c>
       <c r="BE9" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="10" spans="1:57">
@@ -3744,7 +3744,7 @@
         <v>609</v>
       </c>
       <c r="BE10" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="11" spans="1:57">
@@ -3899,7 +3899,7 @@
         <v>609</v>
       </c>
       <c r="BE11" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="12" spans="1:57">
@@ -4051,7 +4051,7 @@
         <v>609</v>
       </c>
       <c r="BE12" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="13" spans="1:57">
@@ -4194,7 +4194,7 @@
         <v>609</v>
       </c>
       <c r="BE13" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="14" spans="1:57">
@@ -4355,7 +4355,7 @@
         <v>609</v>
       </c>
       <c r="BE14" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="15" spans="1:57">
@@ -4510,7 +4510,7 @@
         <v>609</v>
       </c>
       <c r="BE15" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="16" spans="1:57">
@@ -4665,7 +4665,7 @@
         <v>609</v>
       </c>
       <c r="BE16" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="17" spans="1:57">
@@ -4817,7 +4817,7 @@
         <v>609</v>
       </c>
       <c r="BE17" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="18" spans="1:57">
@@ -4969,7 +4969,7 @@
         <v>609</v>
       </c>
       <c r="BE18" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="19" spans="1:57">
@@ -5130,7 +5130,7 @@
         <v>609</v>
       </c>
       <c r="BE19" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="20" spans="1:57">
@@ -5294,7 +5294,7 @@
         <v>609</v>
       </c>
       <c r="BE20" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="21" spans="1:57">
@@ -5446,7 +5446,7 @@
         <v>609</v>
       </c>
       <c r="BE21" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="22" spans="1:57">
@@ -5589,7 +5589,7 @@
         <v>609</v>
       </c>
       <c r="BE22" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="23" spans="1:57">
@@ -5732,7 +5732,7 @@
         <v>609</v>
       </c>
       <c r="BE23" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="24" spans="1:57">
@@ -5893,7 +5893,7 @@
         <v>609</v>
       </c>
       <c r="BE24" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="25" spans="1:57">
@@ -6057,7 +6057,7 @@
         <v>609</v>
       </c>
       <c r="BE25" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="26" spans="1:57">
@@ -6209,7 +6209,7 @@
         <v>609</v>
       </c>
       <c r="BE26" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="27" spans="1:57">
@@ -6358,7 +6358,7 @@
         <v>609</v>
       </c>
       <c r="BE27" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="28" spans="1:57">
@@ -6504,7 +6504,7 @@
         <v>609</v>
       </c>
       <c r="BE28" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="29" spans="1:57">
@@ -6665,7 +6665,7 @@
         <v>609</v>
       </c>
       <c r="BE29" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="30" spans="1:57">
@@ -6808,7 +6808,7 @@
         <v>609</v>
       </c>
       <c r="BE30" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="31" spans="1:57">
@@ -6969,7 +6969,7 @@
         <v>609</v>
       </c>
       <c r="BE31" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="32" spans="1:57">
@@ -7130,7 +7130,7 @@
         <v>609</v>
       </c>
       <c r="BE32" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="33" spans="1:57">
@@ -7291,7 +7291,7 @@
         <v>609</v>
       </c>
       <c r="BE33" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="34" spans="1:57">
@@ -7452,7 +7452,7 @@
         <v>609</v>
       </c>
       <c r="BE34" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="35" spans="1:57">
@@ -7613,7 +7613,7 @@
         <v>609</v>
       </c>
       <c r="BE35" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="36" spans="1:57">
@@ -7777,7 +7777,7 @@
         <v>609</v>
       </c>
       <c r="BE36" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="37" spans="1:57">
@@ -7923,7 +7923,7 @@
         <v>609</v>
       </c>
       <c r="BE37" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="38" spans="1:57">
@@ -8084,7 +8084,7 @@
         <v>609</v>
       </c>
       <c r="BE38" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="39" spans="1:57">
@@ -8245,7 +8245,7 @@
         <v>609</v>
       </c>
       <c r="BE39" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="40" spans="1:57">
@@ -8394,7 +8394,7 @@
         <v>609</v>
       </c>
       <c r="BE40" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="41" spans="1:57">
@@ -8555,7 +8555,7 @@
         <v>609</v>
       </c>
       <c r="BE41" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="42" spans="1:57">
@@ -8698,7 +8698,7 @@
         <v>609</v>
       </c>
       <c r="BE42" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="43" spans="1:57">
@@ -8859,7 +8859,7 @@
         <v>609</v>
       </c>
       <c r="BE43" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="44" spans="1:57">
@@ -9023,7 +9023,7 @@
         <v>609</v>
       </c>
       <c r="BE44" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="45" spans="1:57">
@@ -9169,7 +9169,7 @@
         <v>609</v>
       </c>
       <c r="BE45" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="46" spans="1:57">
@@ -9312,7 +9312,7 @@
         <v>609</v>
       </c>
       <c r="BE46" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="47" spans="1:57">
@@ -9458,7 +9458,7 @@
         <v>609</v>
       </c>
       <c r="BE47" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="48" spans="1:57">
@@ -9622,7 +9622,7 @@
         <v>609</v>
       </c>
       <c r="BE48" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="49" spans="1:57">
@@ -9786,7 +9786,7 @@
         <v>609</v>
       </c>
       <c r="BE49" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="50" spans="1:57">
@@ -9947,7 +9947,7 @@
         <v>609</v>
       </c>
       <c r="BE50" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="51" spans="1:57">
@@ -10096,7 +10096,7 @@
         <v>609</v>
       </c>
       <c r="BE51" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="52" spans="1:57">
@@ -10257,7 +10257,7 @@
         <v>609</v>
       </c>
       <c r="BE52" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="53" spans="1:57">
@@ -10400,7 +10400,7 @@
         <v>609</v>
       </c>
       <c r="BE53" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="54" spans="1:57">
@@ -10561,7 +10561,7 @@
         <v>609</v>
       </c>
       <c r="BE54" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="55" spans="1:57">
@@ -10722,7 +10722,7 @@
         <v>609</v>
       </c>
       <c r="BE55" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="56" spans="1:57">
@@ -10865,7 +10865,7 @@
         <v>609</v>
       </c>
       <c r="BE56" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="57" spans="1:57">
@@ -11026,7 +11026,7 @@
         <v>609</v>
       </c>
       <c r="BE57" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="58" spans="1:57">
@@ -11169,7 +11169,7 @@
         <v>609</v>
       </c>
       <c r="BE58" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="59" spans="1:57">
@@ -11312,7 +11312,7 @@
         <v>609</v>
       </c>
       <c r="BE59" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="60" spans="1:57">
@@ -11455,7 +11455,7 @@
         <v>609</v>
       </c>
       <c r="BE60" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="61" spans="1:57">
@@ -11619,7 +11619,7 @@
         <v>609</v>
       </c>
       <c r="BE61" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="62" spans="1:57">
@@ -11768,7 +11768,7 @@
         <v>609</v>
       </c>
       <c r="BE62" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="63" spans="1:57">
@@ -11911,7 +11911,7 @@
         <v>609</v>
       </c>
       <c r="BE63" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="64" spans="1:57">
@@ -12072,7 +12072,7 @@
         <v>609</v>
       </c>
       <c r="BE64" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="65" spans="1:57">
@@ -12215,7 +12215,7 @@
         <v>609</v>
       </c>
       <c r="BE65" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="66" spans="1:57">
@@ -12358,7 +12358,7 @@
         <v>609</v>
       </c>
       <c r="BE66" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="67" spans="1:57">
@@ -12504,7 +12504,7 @@
         <v>609</v>
       </c>
       <c r="BE67" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="68" spans="1:57">
@@ -12647,7 +12647,7 @@
         <v>609</v>
       </c>
       <c r="BE68" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="69" spans="1:57">
@@ -12790,7 +12790,7 @@
         <v>609</v>
       </c>
       <c r="BE69" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="70" spans="1:57">
@@ -12933,7 +12933,7 @@
         <v>609</v>
       </c>
       <c r="BE70" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="71" spans="1:57">
@@ -13076,7 +13076,7 @@
         <v>609</v>
       </c>
       <c r="BE71" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="72" spans="1:57">
@@ -13237,7 +13237,7 @@
         <v>609</v>
       </c>
       <c r="BE72" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="73" spans="1:57">
@@ -13398,7 +13398,7 @@
         <v>609</v>
       </c>
       <c r="BE73" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="74" spans="1:57">
@@ -13541,7 +13541,7 @@
         <v>609</v>
       </c>
       <c r="BE74" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="75" spans="1:57">
@@ -13684,7 +13684,7 @@
         <v>609</v>
       </c>
       <c r="BE75" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="76" spans="1:57">
@@ -13845,7 +13845,7 @@
         <v>609</v>
       </c>
       <c r="BE76" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="77" spans="1:57">
@@ -14003,7 +14003,7 @@
         <v>609</v>
       </c>
       <c r="BE77" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="78" spans="1:57">
@@ -14146,7 +14146,7 @@
         <v>609</v>
       </c>
       <c r="BE78" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="79" spans="1:57">
@@ -14307,7 +14307,7 @@
         <v>609</v>
       </c>
       <c r="BE79" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="80" spans="1:57">
@@ -14450,7 +14450,7 @@
         <v>609</v>
       </c>
       <c r="BE80" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="81" spans="1:57">
@@ -14611,7 +14611,7 @@
         <v>609</v>
       </c>
       <c r="BE81" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="82" spans="1:57">
@@ -14760,7 +14760,7 @@
         <v>609</v>
       </c>
       <c r="BE82" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="83" spans="1:57">
@@ -14921,7 +14921,7 @@
         <v>609</v>
       </c>
       <c r="BE83" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="84" spans="1:57">
@@ -15067,7 +15067,7 @@
         <v>609</v>
       </c>
       <c r="BE84" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="85" spans="1:57">
@@ -15210,7 +15210,7 @@
         <v>609</v>
       </c>
       <c r="BE85" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="86" spans="1:57">
@@ -15371,7 +15371,7 @@
         <v>609</v>
       </c>
       <c r="BE86" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="87" spans="1:57">
@@ -15517,7 +15517,7 @@
         <v>609</v>
       </c>
       <c r="BE87" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="88" spans="1:57">
@@ -15678,7 +15678,7 @@
         <v>609</v>
       </c>
       <c r="BE88" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="89" spans="1:57">
@@ -15839,7 +15839,7 @@
         <v>609</v>
       </c>
       <c r="BE89" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="90" spans="1:57">
@@ -16000,7 +16000,7 @@
         <v>609</v>
       </c>
       <c r="BE90" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="91" spans="1:57">
@@ -16143,7 +16143,7 @@
         <v>609</v>
       </c>
       <c r="BE91" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="92" spans="1:57">
@@ -16304,7 +16304,7 @@
         <v>609</v>
       </c>
       <c r="BE92" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="93" spans="1:57">
@@ -16447,7 +16447,7 @@
         <v>609</v>
       </c>
       <c r="BE93" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="94" spans="1:57">
@@ -16608,7 +16608,7 @@
         <v>609</v>
       </c>
       <c r="BE94" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="95" spans="1:57">
@@ -16769,7 +16769,7 @@
         <v>609</v>
       </c>
       <c r="BE95" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="96" spans="1:57">
@@ -16921,7 +16921,7 @@
         <v>609</v>
       </c>
       <c r="BE96" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="97" spans="1:57">
@@ -17073,7 +17073,7 @@
         <v>609</v>
       </c>
       <c r="BE97" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="98" spans="1:57">
@@ -17225,7 +17225,7 @@
         <v>609</v>
       </c>
       <c r="BE98" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="99" spans="1:57">
@@ -17377,7 +17377,7 @@
         <v>609</v>
       </c>
       <c r="BE99" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="100" spans="1:57">
@@ -17520,7 +17520,7 @@
         <v>609</v>
       </c>
       <c r="BE100" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="101" spans="1:57">
@@ -17663,7 +17663,7 @@
         <v>609</v>
       </c>
       <c r="BE101" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="102" spans="1:57">
@@ -17806,7 +17806,7 @@
         <v>609</v>
       </c>
       <c r="BE102" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="103" spans="1:57">
@@ -17952,7 +17952,7 @@
         <v>609</v>
       </c>
       <c r="BE103" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="104" spans="1:57">
@@ -18095,7 +18095,7 @@
         <v>609</v>
       </c>
       <c r="BE104" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="105" spans="1:57">
@@ -18253,7 +18253,7 @@
         <v>609</v>
       </c>
       <c r="BE105" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="106" spans="1:57">
@@ -18399,7 +18399,7 @@
         <v>609</v>
       </c>
       <c r="BE106" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="107" spans="1:57">
@@ -18542,7 +18542,7 @@
         <v>609</v>
       </c>
       <c r="BE107" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="108" spans="1:57">
@@ -18688,7 +18688,7 @@
         <v>609</v>
       </c>
       <c r="BE108" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="109" spans="1:57">
@@ -18831,7 +18831,7 @@
         <v>609</v>
       </c>
       <c r="BE109" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="110" spans="1:57">
@@ -18974,7 +18974,7 @@
         <v>609</v>
       </c>
       <c r="BE110" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="111" spans="1:57">
@@ -19117,7 +19117,7 @@
         <v>609</v>
       </c>
       <c r="BE111" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="112" spans="1:57">
@@ -19263,7 +19263,7 @@
         <v>609</v>
       </c>
       <c r="BE112" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="113" spans="1:57">
@@ -19406,7 +19406,7 @@
         <v>609</v>
       </c>
       <c r="BE113" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="114" spans="1:57">
@@ -19552,7 +19552,7 @@
         <v>609</v>
       </c>
       <c r="BE114" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="115" spans="1:57">
@@ -19704,7 +19704,7 @@
         <v>609</v>
       </c>
       <c r="BE115" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="116" spans="1:57">
@@ -19865,7 +19865,7 @@
         <v>609</v>
       </c>
       <c r="BE116" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="117" spans="1:57">
@@ -20008,7 +20008,7 @@
         <v>609</v>
       </c>
       <c r="BE117" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="118" spans="1:57">
@@ -20154,7 +20154,7 @@
         <v>609</v>
       </c>
       <c r="BE118" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="119" spans="1:57">
@@ -20315,7 +20315,7 @@
         <v>609</v>
       </c>
       <c r="BE119" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="120" spans="1:57">
@@ -20476,7 +20476,7 @@
         <v>609</v>
       </c>
       <c r="BE120" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="121" spans="1:57">
@@ -20619,7 +20619,7 @@
         <v>609</v>
       </c>
       <c r="BE121" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="122" spans="1:57">
@@ -20768,7 +20768,7 @@
         <v>609</v>
       </c>
       <c r="BE122" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="123" spans="1:57">
@@ -20911,7 +20911,7 @@
         <v>609</v>
       </c>
       <c r="BE123" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="124" spans="1:57">
@@ -21054,7 +21054,7 @@
         <v>609</v>
       </c>
       <c r="BE124" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="125" spans="1:57">
@@ -21200,7 +21200,7 @@
         <v>609</v>
       </c>
       <c r="BE125" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="126" spans="1:57">
@@ -21343,7 +21343,7 @@
         <v>609</v>
       </c>
       <c r="BE126" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="127" spans="1:57">
@@ -21504,7 +21504,7 @@
         <v>609</v>
       </c>
       <c r="BE127" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="128" spans="1:57">
@@ -21665,7 +21665,7 @@
         <v>609</v>
       </c>
       <c r="BE128" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="129" spans="1:57">
@@ -21808,7 +21808,7 @@
         <v>609</v>
       </c>
       <c r="BE129" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="130" spans="1:57">
@@ -21951,7 +21951,7 @@
         <v>609</v>
       </c>
       <c r="BE130" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="131" spans="1:57">
@@ -22115,7 +22115,7 @@
         <v>609</v>
       </c>
       <c r="BE131" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="132" spans="1:57">
@@ -22258,7 +22258,7 @@
         <v>609</v>
       </c>
       <c r="BE132" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="133" spans="1:57">
@@ -22419,7 +22419,7 @@
         <v>609</v>
       </c>
       <c r="BE133" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="134" spans="1:57">
@@ -22562,7 +22562,7 @@
         <v>609</v>
       </c>
       <c r="BE134" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="135" spans="1:57">
@@ -22723,7 +22723,7 @@
         <v>609</v>
       </c>
       <c r="BE135" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="136" spans="1:57">
@@ -22884,7 +22884,7 @@
         <v>609</v>
       </c>
       <c r="BE136" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="137" spans="1:57">
@@ -23048,7 +23048,7 @@
         <v>609</v>
       </c>
       <c r="BE137" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="138" spans="1:57">
@@ -23209,7 +23209,7 @@
         <v>609</v>
       </c>
       <c r="BE138" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="139" spans="1:57">
@@ -23352,7 +23352,7 @@
         <v>609</v>
       </c>
       <c r="BE139" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="140" spans="1:57">
@@ -23504,7 +23504,7 @@
         <v>609</v>
       </c>
       <c r="BE140" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="141" spans="1:57">
@@ -23647,7 +23647,7 @@
         <v>609</v>
       </c>
       <c r="BE141" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="142" spans="1:57">
@@ -23793,7 +23793,7 @@
         <v>609</v>
       </c>
       <c r="BE142" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="143" spans="1:57">
@@ -23936,7 +23936,7 @@
         <v>609</v>
       </c>
       <c r="BE143" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="144" spans="1:57">
@@ -24085,7 +24085,7 @@
         <v>609</v>
       </c>
       <c r="BE144" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="145" spans="1:57">
@@ -24231,7 +24231,7 @@
         <v>609</v>
       </c>
       <c r="BE145" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="146" spans="1:57">
@@ -24374,7 +24374,7 @@
         <v>609</v>
       </c>
       <c r="BE146" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="147" spans="1:57">
@@ -24517,7 +24517,7 @@
         <v>609</v>
       </c>
       <c r="BE147" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="148" spans="1:57">
@@ -24678,7 +24678,7 @@
         <v>609</v>
       </c>
       <c r="BE148" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="149" spans="1:57">
@@ -24839,7 +24839,7 @@
         <v>609</v>
       </c>
       <c r="BE149" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="150" spans="1:57">
@@ -24985,7 +24985,7 @@
         <v>609</v>
       </c>
       <c r="BE150" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="151" spans="1:57">
@@ -25128,7 +25128,7 @@
         <v>609</v>
       </c>
       <c r="BE151" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="152" spans="1:57">
@@ -25274,7 +25274,7 @@
         <v>609</v>
       </c>
       <c r="BE152" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="153" spans="1:57">
@@ -25420,7 +25420,7 @@
         <v>609</v>
       </c>
       <c r="BE153" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="154" spans="1:57">
@@ -25563,7 +25563,7 @@
         <v>609</v>
       </c>
       <c r="BE154" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="155" spans="1:57">
@@ -25724,7 +25724,7 @@
         <v>609</v>
       </c>
       <c r="BE155" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="156" spans="1:57">
@@ -25873,7 +25873,7 @@
         <v>609</v>
       </c>
       <c r="BE156" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="157" spans="1:57">
@@ -26025,7 +26025,7 @@
         <v>609</v>
       </c>
       <c r="BE157" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="158" spans="1:57">
@@ -26168,7 +26168,7 @@
         <v>609</v>
       </c>
       <c r="BE158" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="159" spans="1:57">
@@ -26329,7 +26329,7 @@
         <v>609</v>
       </c>
       <c r="BE159" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="160" spans="1:57">
@@ -26490,7 +26490,7 @@
         <v>609</v>
       </c>
       <c r="BE160" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="161" spans="1:57">
@@ -26636,7 +26636,7 @@
         <v>609</v>
       </c>
       <c r="BE161" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="162" spans="1:57">
@@ -26782,7 +26782,7 @@
         <v>609</v>
       </c>
       <c r="BE162" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="163" spans="1:57">
@@ -26925,7 +26925,7 @@
         <v>609</v>
       </c>
       <c r="BE163" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="164" spans="1:57">
@@ -27071,7 +27071,7 @@
         <v>609</v>
       </c>
       <c r="BE164" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="165" spans="1:57">
@@ -27232,7 +27232,7 @@
         <v>609</v>
       </c>
       <c r="BE165" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="166" spans="1:57">
@@ -27387,7 +27387,7 @@
         <v>609</v>
       </c>
       <c r="BE166" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="167" spans="1:57">
@@ -27530,7 +27530,7 @@
         <v>609</v>
       </c>
       <c r="BE167" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="168" spans="1:57">
@@ -27682,7 +27682,7 @@
         <v>609</v>
       </c>
       <c r="BE168" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="169" spans="1:57">
@@ -27828,7 +27828,7 @@
         <v>609</v>
       </c>
       <c r="BE169" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="170" spans="1:57">
@@ -27971,7 +27971,7 @@
         <v>609</v>
       </c>
       <c r="BE170" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="171" spans="1:57">
@@ -28135,7 +28135,7 @@
         <v>609</v>
       </c>
       <c r="BE171" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="172" spans="1:57">
@@ -28278,7 +28278,7 @@
         <v>609</v>
       </c>
       <c r="BE172" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="173" spans="1:57">
@@ -28421,7 +28421,7 @@
         <v>609</v>
       </c>
       <c r="BE173" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="174" spans="1:57">
@@ -28588,7 +28588,7 @@
         <v>609</v>
       </c>
       <c r="BE174" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="175" spans="1:57">
@@ -28749,7 +28749,7 @@
         <v>609</v>
       </c>
       <c r="BE175" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="176" spans="1:57">
@@ -28910,7 +28910,7 @@
         <v>609</v>
       </c>
       <c r="BE176" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="177" spans="1:57">
@@ -29053,7 +29053,7 @@
         <v>609</v>
       </c>
       <c r="BE177" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="178" spans="1:57">
@@ -29196,7 +29196,7 @@
         <v>609</v>
       </c>
       <c r="BE178" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="179" spans="1:57">
@@ -29342,7 +29342,7 @@
         <v>609</v>
       </c>
       <c r="BE179" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="180" spans="1:57">
@@ -29485,7 +29485,7 @@
         <v>609</v>
       </c>
       <c r="BE180" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="181" spans="1:57">
@@ -29646,7 +29646,7 @@
         <v>609</v>
       </c>
       <c r="BE181" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="182" spans="1:57">
@@ -29795,7 +29795,7 @@
         <v>609</v>
       </c>
       <c r="BE182" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="183" spans="1:57">
@@ -29941,7 +29941,7 @@
         <v>609</v>
       </c>
       <c r="BE183" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="184" spans="1:57">
@@ -30087,7 +30087,7 @@
         <v>609</v>
       </c>
       <c r="BE184" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="185" spans="1:57">
@@ -30230,7 +30230,7 @@
         <v>609</v>
       </c>
       <c r="BE185" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="186" spans="1:57">
@@ -30376,7 +30376,7 @@
         <v>609</v>
       </c>
       <c r="BE186" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="187" spans="1:57">
@@ -30522,7 +30522,7 @@
         <v>609</v>
       </c>
       <c r="BE187" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="188" spans="1:57">
@@ -30665,7 +30665,7 @@
         <v>609</v>
       </c>
       <c r="BE188" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="189" spans="1:57">
@@ -30808,7 +30808,7 @@
         <v>609</v>
       </c>
       <c r="BE189" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="190" spans="1:57">
@@ -30951,7 +30951,7 @@
         <v>609</v>
       </c>
       <c r="BE190" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="191" spans="1:57">
@@ -31112,7 +31112,7 @@
         <v>609</v>
       </c>
       <c r="BE191" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="192" spans="1:57">
@@ -31258,7 +31258,7 @@
         <v>609</v>
       </c>
       <c r="BE192" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="193" spans="1:57">
@@ -31407,7 +31407,7 @@
         <v>609</v>
       </c>
       <c r="BE193" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="194" spans="1:57">
@@ -31550,7 +31550,7 @@
         <v>609</v>
       </c>
       <c r="BE194" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="195" spans="1:57">
@@ -31693,7 +31693,7 @@
         <v>609</v>
       </c>
       <c r="BE195" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="196" spans="1:57">
@@ -31836,7 +31836,7 @@
         <v>609</v>
       </c>
       <c r="BE196" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="197" spans="1:57">
@@ -31979,7 +31979,7 @@
         <v>609</v>
       </c>
       <c r="BE197" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="198" spans="1:57">
@@ -32125,7 +32125,7 @@
         <v>609</v>
       </c>
       <c r="BE198" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="199" spans="1:57">
@@ -32286,7 +32286,7 @@
         <v>609</v>
       </c>
       <c r="BE199" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="200" spans="1:57">
@@ -32432,7 +32432,7 @@
         <v>609</v>
       </c>
       <c r="BE200" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="201" spans="1:57">
@@ -32584,7 +32584,7 @@
         <v>609</v>
       </c>
       <c r="BE201" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="202" spans="1:57">
@@ -32745,7 +32745,7 @@
         <v>609</v>
       </c>
       <c r="BE202" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="203" spans="1:57">
@@ -32906,7 +32906,7 @@
         <v>609</v>
       </c>
       <c r="BE203" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="204" spans="1:57">
@@ -33067,7 +33067,7 @@
         <v>609</v>
       </c>
       <c r="BE204" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="205" spans="1:57">
@@ -33210,7 +33210,7 @@
         <v>609</v>
       </c>
       <c r="BE205" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="206" spans="1:57">
@@ -33356,7 +33356,7 @@
         <v>609</v>
       </c>
       <c r="BE206" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="207" spans="1:57">
@@ -33499,7 +33499,7 @@
         <v>609</v>
       </c>
       <c r="BE207" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="208" spans="1:57">
@@ -33642,7 +33642,7 @@
         <v>609</v>
       </c>
       <c r="BE208" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
     <row r="209" spans="1:57">
@@ -33785,7 +33785,7 @@
         <v>609</v>
       </c>
       <c r="BE209" s="2">
-        <v>46042.0965728616</v>
+        <v>46042.11739075781</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily dashboard refresh 2026-01-20 07:05
</commit_message>
<xml_diff>
--- a/data/Fail.xlsx
+++ b/data/Fail.xlsx
@@ -2488,7 +2488,7 @@
         <v>589</v>
       </c>
       <c r="BE2" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="3" spans="1:57">
@@ -2631,7 +2631,7 @@
         <v>589</v>
       </c>
       <c r="BE3" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="4" spans="1:57">
@@ -2792,7 +2792,7 @@
         <v>589</v>
       </c>
       <c r="BE4" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="5" spans="1:57">
@@ -2956,7 +2956,7 @@
         <v>589</v>
       </c>
       <c r="BE5" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="6" spans="1:57">
@@ -3117,7 +3117,7 @@
         <v>589</v>
       </c>
       <c r="BE6" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="7" spans="1:57">
@@ -3272,7 +3272,7 @@
         <v>589</v>
       </c>
       <c r="BE7" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="8" spans="1:57">
@@ -3433,7 +3433,7 @@
         <v>589</v>
       </c>
       <c r="BE8" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="9" spans="1:57">
@@ -3576,7 +3576,7 @@
         <v>589</v>
       </c>
       <c r="BE9" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="10" spans="1:57">
@@ -3719,7 +3719,7 @@
         <v>589</v>
       </c>
       <c r="BE10" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="11" spans="1:57">
@@ -3865,7 +3865,7 @@
         <v>589</v>
       </c>
       <c r="BE11" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="12" spans="1:57">
@@ -4026,7 +4026,7 @@
         <v>589</v>
       </c>
       <c r="BE12" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="13" spans="1:57">
@@ -4187,7 +4187,7 @@
         <v>589</v>
       </c>
       <c r="BE13" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="14" spans="1:57">
@@ -4348,7 +4348,7 @@
         <v>589</v>
       </c>
       <c r="BE14" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="15" spans="1:57">
@@ -4497,7 +4497,7 @@
         <v>589</v>
       </c>
       <c r="BE15" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="16" spans="1:57">
@@ -4658,7 +4658,7 @@
         <v>589</v>
       </c>
       <c r="BE16" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="17" spans="1:57">
@@ -4807,7 +4807,7 @@
         <v>589</v>
       </c>
       <c r="BE17" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="18" spans="1:57">
@@ -4950,7 +4950,7 @@
         <v>589</v>
       </c>
       <c r="BE18" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="19" spans="1:57">
@@ -5111,7 +5111,7 @@
         <v>589</v>
       </c>
       <c r="BE19" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="20" spans="1:57">
@@ -5272,7 +5272,7 @@
         <v>589</v>
       </c>
       <c r="BE20" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="21" spans="1:57">
@@ -5433,7 +5433,7 @@
         <v>589</v>
       </c>
       <c r="BE21" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="22" spans="1:57">
@@ -5585,7 +5585,7 @@
         <v>589</v>
       </c>
       <c r="BE22" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="23" spans="1:57">
@@ -5731,7 +5731,7 @@
         <v>589</v>
       </c>
       <c r="BE23" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="24" spans="1:57">
@@ -5892,7 +5892,7 @@
         <v>589</v>
       </c>
       <c r="BE24" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="25" spans="1:57">
@@ -6035,7 +6035,7 @@
         <v>589</v>
       </c>
       <c r="BE25" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="26" spans="1:57">
@@ -6196,7 +6196,7 @@
         <v>589</v>
       </c>
       <c r="BE26" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="27" spans="1:57">
@@ -6339,7 +6339,7 @@
         <v>589</v>
       </c>
       <c r="BE27" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="28" spans="1:57">
@@ -6482,7 +6482,7 @@
         <v>589</v>
       </c>
       <c r="BE28" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="29" spans="1:57">
@@ -6625,7 +6625,7 @@
         <v>589</v>
       </c>
       <c r="BE29" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="30" spans="1:57">
@@ -6786,7 +6786,7 @@
         <v>589</v>
       </c>
       <c r="BE30" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="31" spans="1:57">
@@ -6932,7 +6932,7 @@
         <v>589</v>
       </c>
       <c r="BE31" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="32" spans="1:57">
@@ -7078,7 +7078,7 @@
         <v>589</v>
       </c>
       <c r="BE32" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="33" spans="1:57">
@@ -7230,7 +7230,7 @@
         <v>589</v>
       </c>
       <c r="BE33" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="34" spans="1:57">
@@ -7376,7 +7376,7 @@
         <v>589</v>
       </c>
       <c r="BE34" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="35" spans="1:57">
@@ -7528,7 +7528,7 @@
         <v>589</v>
       </c>
       <c r="BE35" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="36" spans="1:57">
@@ -7671,7 +7671,7 @@
         <v>589</v>
       </c>
       <c r="BE36" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="37" spans="1:57">
@@ -7814,7 +7814,7 @@
         <v>589</v>
       </c>
       <c r="BE37" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="38" spans="1:57">
@@ -7975,7 +7975,7 @@
         <v>589</v>
       </c>
       <c r="BE38" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="39" spans="1:57">
@@ -8121,7 +8121,7 @@
         <v>589</v>
       </c>
       <c r="BE39" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="40" spans="1:57">
@@ -8267,7 +8267,7 @@
         <v>589</v>
       </c>
       <c r="BE40" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="41" spans="1:57">
@@ -8419,7 +8419,7 @@
         <v>589</v>
       </c>
       <c r="BE41" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="42" spans="1:57">
@@ -8562,7 +8562,7 @@
         <v>589</v>
       </c>
       <c r="BE42" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="43" spans="1:57">
@@ -8723,7 +8723,7 @@
         <v>589</v>
       </c>
       <c r="BE43" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="44" spans="1:57">
@@ -8869,7 +8869,7 @@
         <v>589</v>
       </c>
       <c r="BE44" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="45" spans="1:57">
@@ -9024,7 +9024,7 @@
         <v>589</v>
       </c>
       <c r="BE45" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="46" spans="1:57">
@@ -9167,7 +9167,7 @@
         <v>589</v>
       </c>
       <c r="BE46" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="47" spans="1:57">
@@ -9328,7 +9328,7 @@
         <v>589</v>
       </c>
       <c r="BE47" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="48" spans="1:57">
@@ -9471,7 +9471,7 @@
         <v>589</v>
       </c>
       <c r="BE48" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="49" spans="1:57">
@@ -9623,7 +9623,7 @@
         <v>589</v>
       </c>
       <c r="BE49" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="50" spans="1:57">
@@ -9775,7 +9775,7 @@
         <v>589</v>
       </c>
       <c r="BE50" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="51" spans="1:57">
@@ -9924,7 +9924,7 @@
         <v>589</v>
       </c>
       <c r="BE51" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="52" spans="1:57">
@@ -10067,7 +10067,7 @@
         <v>589</v>
       </c>
       <c r="BE52" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="53" spans="1:57">
@@ -10210,7 +10210,7 @@
         <v>589</v>
       </c>
       <c r="BE53" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="54" spans="1:57">
@@ -10353,7 +10353,7 @@
         <v>589</v>
       </c>
       <c r="BE54" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="55" spans="1:57">
@@ -10505,7 +10505,7 @@
         <v>589</v>
       </c>
       <c r="BE55" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="56" spans="1:57">
@@ -10657,7 +10657,7 @@
         <v>589</v>
       </c>
       <c r="BE56" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="57" spans="1:57">
@@ -10818,7 +10818,7 @@
         <v>589</v>
       </c>
       <c r="BE57" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="58" spans="1:57">
@@ -10961,7 +10961,7 @@
         <v>589</v>
       </c>
       <c r="BE58" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="59" spans="1:57">
@@ -11104,7 +11104,7 @@
         <v>589</v>
       </c>
       <c r="BE59" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="60" spans="1:57">
@@ -11265,7 +11265,7 @@
         <v>589</v>
       </c>
       <c r="BE60" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="61" spans="1:57">
@@ -11426,7 +11426,7 @@
         <v>589</v>
       </c>
       <c r="BE61" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="62" spans="1:57">
@@ -11572,7 +11572,7 @@
         <v>589</v>
       </c>
       <c r="BE62" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="63" spans="1:57">
@@ -11718,7 +11718,7 @@
         <v>589</v>
       </c>
       <c r="BE63" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="64" spans="1:57">
@@ -11864,7 +11864,7 @@
         <v>589</v>
       </c>
       <c r="BE64" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="65" spans="1:57">
@@ -12016,7 +12016,7 @@
         <v>589</v>
       </c>
       <c r="BE65" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="66" spans="1:57">
@@ -12177,7 +12177,7 @@
         <v>589</v>
       </c>
       <c r="BE66" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="67" spans="1:57">
@@ -12338,7 +12338,7 @@
         <v>589</v>
       </c>
       <c r="BE67" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="68" spans="1:57">
@@ -12499,7 +12499,7 @@
         <v>589</v>
       </c>
       <c r="BE68" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="69" spans="1:57">
@@ -12660,7 +12660,7 @@
         <v>589</v>
       </c>
       <c r="BE69" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="70" spans="1:57">
@@ -12806,7 +12806,7 @@
         <v>589</v>
       </c>
       <c r="BE70" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="71" spans="1:57">
@@ -12955,7 +12955,7 @@
         <v>589</v>
       </c>
       <c r="BE71" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="72" spans="1:57">
@@ -13101,7 +13101,7 @@
         <v>589</v>
       </c>
       <c r="BE72" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="73" spans="1:57">
@@ -13256,7 +13256,7 @@
         <v>589</v>
       </c>
       <c r="BE73" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="74" spans="1:57">
@@ -13411,7 +13411,7 @@
         <v>589</v>
       </c>
       <c r="BE74" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="75" spans="1:57">
@@ -13569,7 +13569,7 @@
         <v>589</v>
       </c>
       <c r="BE75" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="76" spans="1:57">
@@ -13730,7 +13730,7 @@
         <v>589</v>
       </c>
       <c r="BE76" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="77" spans="1:57">
@@ -13891,7 +13891,7 @@
         <v>589</v>
       </c>
       <c r="BE77" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="78" spans="1:57">
@@ -14052,7 +14052,7 @@
         <v>589</v>
       </c>
       <c r="BE78" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="79" spans="1:57">
@@ -14213,7 +14213,7 @@
         <v>589</v>
       </c>
       <c r="BE79" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="80" spans="1:57">
@@ -14374,7 +14374,7 @@
         <v>589</v>
       </c>
       <c r="BE80" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="81" spans="1:57">
@@ -14517,7 +14517,7 @@
         <v>589</v>
       </c>
       <c r="BE81" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="82" spans="1:57">
@@ -14678,7 +14678,7 @@
         <v>589</v>
       </c>
       <c r="BE82" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="83" spans="1:57">
@@ -14821,7 +14821,7 @@
         <v>589</v>
       </c>
       <c r="BE83" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="84" spans="1:57">
@@ -14973,7 +14973,7 @@
         <v>589</v>
       </c>
       <c r="BE84" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="85" spans="1:57">
@@ -15116,7 +15116,7 @@
         <v>589</v>
       </c>
       <c r="BE85" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="86" spans="1:57">
@@ -15259,7 +15259,7 @@
         <v>589</v>
       </c>
       <c r="BE86" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="87" spans="1:57">
@@ -15405,7 +15405,7 @@
         <v>589</v>
       </c>
       <c r="BE87" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="88" spans="1:57">
@@ -15572,7 +15572,7 @@
         <v>589</v>
       </c>
       <c r="BE88" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="89" spans="1:57">
@@ -15718,7 +15718,7 @@
         <v>589</v>
       </c>
       <c r="BE89" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="90" spans="1:57">
@@ -15879,7 +15879,7 @@
         <v>589</v>
       </c>
       <c r="BE90" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="91" spans="1:57">
@@ -16022,7 +16022,7 @@
         <v>589</v>
       </c>
       <c r="BE91" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="92" spans="1:57">
@@ -16168,7 +16168,7 @@
         <v>589</v>
       </c>
       <c r="BE92" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="93" spans="1:57">
@@ -16314,7 +16314,7 @@
         <v>589</v>
       </c>
       <c r="BE93" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="94" spans="1:57">
@@ -16457,7 +16457,7 @@
         <v>589</v>
       </c>
       <c r="BE94" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="95" spans="1:57">
@@ -16600,7 +16600,7 @@
         <v>589</v>
       </c>
       <c r="BE95" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="96" spans="1:57">
@@ -16743,7 +16743,7 @@
         <v>589</v>
       </c>
       <c r="BE96" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="97" spans="1:57">
@@ -16889,7 +16889,7 @@
         <v>589</v>
       </c>
       <c r="BE97" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="98" spans="1:57">
@@ -17041,7 +17041,7 @@
         <v>589</v>
       </c>
       <c r="BE98" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="99" spans="1:57">
@@ -17184,7 +17184,7 @@
         <v>589</v>
       </c>
       <c r="BE99" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="100" spans="1:57">
@@ -17327,7 +17327,7 @@
         <v>589</v>
       </c>
       <c r="BE100" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="101" spans="1:57">
@@ -17491,7 +17491,7 @@
         <v>589</v>
       </c>
       <c r="BE101" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="102" spans="1:57">
@@ -17634,7 +17634,7 @@
         <v>589</v>
       </c>
       <c r="BE102" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="103" spans="1:57">
@@ -17777,7 +17777,7 @@
         <v>589</v>
       </c>
       <c r="BE103" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="104" spans="1:57">
@@ -17938,7 +17938,7 @@
         <v>589</v>
       </c>
       <c r="BE104" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="105" spans="1:57">
@@ -18099,7 +18099,7 @@
         <v>589</v>
       </c>
       <c r="BE105" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="106" spans="1:57">
@@ -18260,7 +18260,7 @@
         <v>589</v>
       </c>
       <c r="BE106" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="107" spans="1:57">
@@ -18421,7 +18421,7 @@
         <v>589</v>
       </c>
       <c r="BE107" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="108" spans="1:57">
@@ -18582,7 +18582,7 @@
         <v>589</v>
       </c>
       <c r="BE108" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="109" spans="1:57">
@@ -18731,7 +18731,7 @@
         <v>589</v>
       </c>
       <c r="BE109" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="110" spans="1:57">
@@ -18874,7 +18874,7 @@
         <v>589</v>
       </c>
       <c r="BE110" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="111" spans="1:57">
@@ -19038,7 +19038,7 @@
         <v>589</v>
       </c>
       <c r="BE111" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="112" spans="1:57">
@@ -19181,7 +19181,7 @@
         <v>589</v>
       </c>
       <c r="BE112" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="113" spans="1:57">
@@ -19327,7 +19327,7 @@
         <v>589</v>
       </c>
       <c r="BE113" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="114" spans="1:57">
@@ -19470,7 +19470,7 @@
         <v>589</v>
       </c>
       <c r="BE114" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="115" spans="1:57">
@@ -19613,7 +19613,7 @@
         <v>589</v>
       </c>
       <c r="BE115" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="116" spans="1:57">
@@ -19759,7 +19759,7 @@
         <v>589</v>
       </c>
       <c r="BE116" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="117" spans="1:57">
@@ -19920,7 +19920,7 @@
         <v>589</v>
       </c>
       <c r="BE117" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="118" spans="1:57">
@@ -20069,7 +20069,7 @@
         <v>589</v>
       </c>
       <c r="BE118" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="119" spans="1:57">
@@ -20218,7 +20218,7 @@
         <v>589</v>
       </c>
       <c r="BE119" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="120" spans="1:57">
@@ -20361,7 +20361,7 @@
         <v>589</v>
       </c>
       <c r="BE120" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="121" spans="1:57">
@@ -20504,7 +20504,7 @@
         <v>589</v>
       </c>
       <c r="BE121" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="122" spans="1:57">
@@ -20650,7 +20650,7 @@
         <v>589</v>
       </c>
       <c r="BE122" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="123" spans="1:57">
@@ -20811,7 +20811,7 @@
         <v>589</v>
       </c>
       <c r="BE123" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="124" spans="1:57">
@@ -20972,7 +20972,7 @@
         <v>589</v>
       </c>
       <c r="BE124" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="125" spans="1:57">
@@ -21115,7 +21115,7 @@
         <v>589</v>
       </c>
       <c r="BE125" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="126" spans="1:57">
@@ -21276,7 +21276,7 @@
         <v>589</v>
       </c>
       <c r="BE126" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="127" spans="1:57">
@@ -21425,7 +21425,7 @@
         <v>589</v>
       </c>
       <c r="BE127" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="128" spans="1:57">
@@ -21568,7 +21568,7 @@
         <v>589</v>
       </c>
       <c r="BE128" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="129" spans="1:57">
@@ -21711,7 +21711,7 @@
         <v>589</v>
       </c>
       <c r="BE129" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="130" spans="1:57">
@@ -21854,7 +21854,7 @@
         <v>589</v>
       </c>
       <c r="BE130" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="131" spans="1:57">
@@ -21997,7 +21997,7 @@
         <v>589</v>
       </c>
       <c r="BE131" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="132" spans="1:57">
@@ -22146,7 +22146,7 @@
         <v>589</v>
       </c>
       <c r="BE132" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="133" spans="1:57">
@@ -22289,7 +22289,7 @@
         <v>589</v>
       </c>
       <c r="BE133" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="134" spans="1:57">
@@ -22435,7 +22435,7 @@
         <v>589</v>
       </c>
       <c r="BE134" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="135" spans="1:57">
@@ -22578,7 +22578,7 @@
         <v>589</v>
       </c>
       <c r="BE135" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="136" spans="1:57">
@@ -22721,7 +22721,7 @@
         <v>589</v>
       </c>
       <c r="BE136" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="137" spans="1:57">
@@ -22885,7 +22885,7 @@
         <v>589</v>
       </c>
       <c r="BE137" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="138" spans="1:57">
@@ -23028,7 +23028,7 @@
         <v>589</v>
       </c>
       <c r="BE138" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="139" spans="1:57">
@@ -23189,7 +23189,7 @@
         <v>589</v>
       </c>
       <c r="BE139" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="140" spans="1:57">
@@ -23332,7 +23332,7 @@
         <v>589</v>
       </c>
       <c r="BE140" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="141" spans="1:57">
@@ -23475,7 +23475,7 @@
         <v>589</v>
       </c>
       <c r="BE141" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="142" spans="1:57">
@@ -23627,7 +23627,7 @@
         <v>589</v>
       </c>
       <c r="BE142" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="143" spans="1:57">
@@ -23773,7 +23773,7 @@
         <v>589</v>
       </c>
       <c r="BE143" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="144" spans="1:57">
@@ -23919,7 +23919,7 @@
         <v>589</v>
       </c>
       <c r="BE144" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="145" spans="1:57">
@@ -24062,7 +24062,7 @@
         <v>589</v>
       </c>
       <c r="BE145" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="146" spans="1:57">
@@ -24211,7 +24211,7 @@
         <v>589</v>
       </c>
       <c r="BE146" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="147" spans="1:57">
@@ -24357,7 +24357,7 @@
         <v>589</v>
       </c>
       <c r="BE147" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="148" spans="1:57">
@@ -24500,7 +24500,7 @@
         <v>589</v>
       </c>
       <c r="BE148" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="149" spans="1:57">
@@ -24643,7 +24643,7 @@
         <v>589</v>
       </c>
       <c r="BE149" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="150" spans="1:57">
@@ -24804,7 +24804,7 @@
         <v>589</v>
       </c>
       <c r="BE150" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="151" spans="1:57">
@@ -24965,7 +24965,7 @@
         <v>589</v>
       </c>
       <c r="BE151" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="152" spans="1:57">
@@ -25126,7 +25126,7 @@
         <v>589</v>
       </c>
       <c r="BE152" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="153" spans="1:57">
@@ -25287,7 +25287,7 @@
         <v>589</v>
       </c>
       <c r="BE153" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="154" spans="1:57">
@@ -25433,7 +25433,7 @@
         <v>589</v>
       </c>
       <c r="BE154" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="155" spans="1:57">
@@ -25576,7 +25576,7 @@
         <v>589</v>
       </c>
       <c r="BE155" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="156" spans="1:57">
@@ -25728,7 +25728,7 @@
         <v>589</v>
       </c>
       <c r="BE156" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="157" spans="1:57">
@@ -25889,7 +25889,7 @@
         <v>589</v>
       </c>
       <c r="BE157" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="158" spans="1:57">
@@ -26032,7 +26032,7 @@
         <v>589</v>
       </c>
       <c r="BE158" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="159" spans="1:57">
@@ -26181,7 +26181,7 @@
         <v>589</v>
       </c>
       <c r="BE159" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="160" spans="1:57">
@@ -26324,7 +26324,7 @@
         <v>589</v>
       </c>
       <c r="BE160" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="161" spans="1:57">
@@ -26485,7 +26485,7 @@
         <v>589</v>
       </c>
       <c r="BE161" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="162" spans="1:57">
@@ -26631,7 +26631,7 @@
         <v>589</v>
       </c>
       <c r="BE162" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="163" spans="1:57">
@@ -26774,7 +26774,7 @@
         <v>589</v>
       </c>
       <c r="BE163" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="164" spans="1:57">
@@ -26938,7 +26938,7 @@
         <v>589</v>
       </c>
       <c r="BE164" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="165" spans="1:57">
@@ -27084,7 +27084,7 @@
         <v>589</v>
       </c>
       <c r="BE165" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="166" spans="1:57">
@@ -27236,7 +27236,7 @@
         <v>589</v>
       </c>
       <c r="BE166" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="167" spans="1:57">
@@ -27388,7 +27388,7 @@
         <v>589</v>
       </c>
       <c r="BE167" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="168" spans="1:57">
@@ -27549,7 +27549,7 @@
         <v>589</v>
       </c>
       <c r="BE168" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="169" spans="1:57">
@@ -27713,7 +27713,7 @@
         <v>589</v>
       </c>
       <c r="BE169" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="170" spans="1:57">
@@ -27874,7 +27874,7 @@
         <v>589</v>
       </c>
       <c r="BE170" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="171" spans="1:57">
@@ -28026,7 +28026,7 @@
         <v>589</v>
       </c>
       <c r="BE171" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="172" spans="1:57">
@@ -28169,7 +28169,7 @@
         <v>589</v>
       </c>
       <c r="BE172" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="173" spans="1:57">
@@ -28312,7 +28312,7 @@
         <v>589</v>
       </c>
       <c r="BE173" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="174" spans="1:57">
@@ -28473,7 +28473,7 @@
         <v>589</v>
       </c>
       <c r="BE174" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="175" spans="1:57">
@@ -28616,7 +28616,7 @@
         <v>589</v>
       </c>
       <c r="BE175" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="176" spans="1:57">
@@ -28759,7 +28759,7 @@
         <v>589</v>
       </c>
       <c r="BE176" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="177" spans="1:57">
@@ -28902,7 +28902,7 @@
         <v>589</v>
       </c>
       <c r="BE177" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="178" spans="1:57">
@@ -29045,7 +29045,7 @@
         <v>589</v>
       </c>
       <c r="BE178" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
     <row r="179" spans="1:57">
@@ -29206,7 +29206,7 @@
         <v>589</v>
       </c>
       <c r="BE179" s="2">
-        <v>46042.12719424296</v>
+        <v>46042.29230409503</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily dashboard refresh 2026-01-22 21:08
</commit_message>
<xml_diff>
--- a/data/Fail.xlsx
+++ b/data/Fail.xlsx
@@ -2536,7 +2536,7 @@
         <v>605</v>
       </c>
       <c r="BE2" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="3" spans="1:57">
@@ -2679,7 +2679,7 @@
         <v>605</v>
       </c>
       <c r="BE3" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="4" spans="1:57">
@@ -2840,7 +2840,7 @@
         <v>605</v>
       </c>
       <c r="BE4" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="5" spans="1:57">
@@ -3004,7 +3004,7 @@
         <v>605</v>
       </c>
       <c r="BE5" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="6" spans="1:57">
@@ -3165,7 +3165,7 @@
         <v>605</v>
       </c>
       <c r="BE6" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="7" spans="1:57">
@@ -3320,7 +3320,7 @@
         <v>605</v>
       </c>
       <c r="BE7" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="8" spans="1:57">
@@ -3481,7 +3481,7 @@
         <v>605</v>
       </c>
       <c r="BE8" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="9" spans="1:57">
@@ -3624,7 +3624,7 @@
         <v>605</v>
       </c>
       <c r="BE9" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="10" spans="1:57">
@@ -3767,7 +3767,7 @@
         <v>605</v>
       </c>
       <c r="BE10" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="11" spans="1:57">
@@ -3913,7 +3913,7 @@
         <v>605</v>
       </c>
       <c r="BE11" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="12" spans="1:57">
@@ -4074,7 +4074,7 @@
         <v>605</v>
       </c>
       <c r="BE12" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="13" spans="1:57">
@@ -4235,7 +4235,7 @@
         <v>605</v>
       </c>
       <c r="BE13" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="14" spans="1:57">
@@ -4396,7 +4396,7 @@
         <v>605</v>
       </c>
       <c r="BE14" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="15" spans="1:57">
@@ -4545,7 +4545,7 @@
         <v>605</v>
       </c>
       <c r="BE15" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="16" spans="1:57">
@@ -4706,7 +4706,7 @@
         <v>605</v>
       </c>
       <c r="BE16" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="17" spans="1:57">
@@ -4852,7 +4852,7 @@
         <v>605</v>
       </c>
       <c r="BE17" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="18" spans="1:57">
@@ -4995,7 +4995,7 @@
         <v>605</v>
       </c>
       <c r="BE18" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="19" spans="1:57">
@@ -5156,7 +5156,7 @@
         <v>605</v>
       </c>
       <c r="BE19" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="20" spans="1:57">
@@ -5317,7 +5317,7 @@
         <v>605</v>
       </c>
       <c r="BE20" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="21" spans="1:57">
@@ -5478,7 +5478,7 @@
         <v>605</v>
       </c>
       <c r="BE21" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="22" spans="1:57">
@@ -5630,7 +5630,7 @@
         <v>605</v>
       </c>
       <c r="BE22" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="23" spans="1:57">
@@ -5776,7 +5776,7 @@
         <v>605</v>
       </c>
       <c r="BE23" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="24" spans="1:57">
@@ -5937,7 +5937,7 @@
         <v>605</v>
       </c>
       <c r="BE24" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="25" spans="1:57">
@@ -6080,7 +6080,7 @@
         <v>605</v>
       </c>
       <c r="BE25" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="26" spans="1:57">
@@ -6241,7 +6241,7 @@
         <v>605</v>
       </c>
       <c r="BE26" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="27" spans="1:57">
@@ -6384,7 +6384,7 @@
         <v>605</v>
       </c>
       <c r="BE27" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="28" spans="1:57">
@@ -6527,7 +6527,7 @@
         <v>605</v>
       </c>
       <c r="BE28" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="29" spans="1:57">
@@ -6670,7 +6670,7 @@
         <v>605</v>
       </c>
       <c r="BE29" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="30" spans="1:57">
@@ -6813,7 +6813,7 @@
         <v>605</v>
       </c>
       <c r="BE30" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="31" spans="1:57">
@@ -6974,7 +6974,7 @@
         <v>605</v>
       </c>
       <c r="BE31" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="32" spans="1:57">
@@ -7120,7 +7120,7 @@
         <v>605</v>
       </c>
       <c r="BE32" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="33" spans="1:57">
@@ -7266,7 +7266,7 @@
         <v>605</v>
       </c>
       <c r="BE33" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="34" spans="1:57">
@@ -7418,7 +7418,7 @@
         <v>605</v>
       </c>
       <c r="BE34" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="35" spans="1:57">
@@ -7564,7 +7564,7 @@
         <v>605</v>
       </c>
       <c r="BE35" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="36" spans="1:57">
@@ -7716,7 +7716,7 @@
         <v>605</v>
       </c>
       <c r="BE36" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="37" spans="1:57">
@@ -7859,7 +7859,7 @@
         <v>605</v>
       </c>
       <c r="BE37" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="38" spans="1:57">
@@ -8002,7 +8002,7 @@
         <v>605</v>
       </c>
       <c r="BE38" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="39" spans="1:57">
@@ -8163,7 +8163,7 @@
         <v>605</v>
       </c>
       <c r="BE39" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="40" spans="1:57">
@@ -8306,7 +8306,7 @@
         <v>605</v>
       </c>
       <c r="BE40" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="41" spans="1:57">
@@ -8452,7 +8452,7 @@
         <v>605</v>
       </c>
       <c r="BE41" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="42" spans="1:57">
@@ -8604,7 +8604,7 @@
         <v>605</v>
       </c>
       <c r="BE42" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="43" spans="1:57">
@@ -8747,7 +8747,7 @@
         <v>605</v>
       </c>
       <c r="BE43" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="44" spans="1:57">
@@ -8908,7 +8908,7 @@
         <v>605</v>
       </c>
       <c r="BE44" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="45" spans="1:57">
@@ -9054,7 +9054,7 @@
         <v>605</v>
       </c>
       <c r="BE45" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="46" spans="1:57">
@@ -9209,7 +9209,7 @@
         <v>605</v>
       </c>
       <c r="BE46" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="47" spans="1:57">
@@ -9352,7 +9352,7 @@
         <v>605</v>
       </c>
       <c r="BE47" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="48" spans="1:57">
@@ -9513,7 +9513,7 @@
         <v>605</v>
       </c>
       <c r="BE48" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="49" spans="1:57">
@@ -9656,7 +9656,7 @@
         <v>605</v>
       </c>
       <c r="BE49" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="50" spans="1:57">
@@ -9808,7 +9808,7 @@
         <v>605</v>
       </c>
       <c r="BE50" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="51" spans="1:57">
@@ -9960,7 +9960,7 @@
         <v>605</v>
       </c>
       <c r="BE51" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="52" spans="1:57">
@@ -10109,7 +10109,7 @@
         <v>605</v>
       </c>
       <c r="BE52" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="53" spans="1:57">
@@ -10252,7 +10252,7 @@
         <v>605</v>
       </c>
       <c r="BE53" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="54" spans="1:57">
@@ -10395,7 +10395,7 @@
         <v>605</v>
       </c>
       <c r="BE54" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="55" spans="1:57">
@@ -10538,7 +10538,7 @@
         <v>605</v>
       </c>
       <c r="BE55" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="56" spans="1:57">
@@ -10690,7 +10690,7 @@
         <v>605</v>
       </c>
       <c r="BE56" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="57" spans="1:57">
@@ -10842,7 +10842,7 @@
         <v>605</v>
       </c>
       <c r="BE57" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="58" spans="1:57">
@@ -11003,7 +11003,7 @@
         <v>605</v>
       </c>
       <c r="BE58" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="59" spans="1:57">
@@ -11146,7 +11146,7 @@
         <v>605</v>
       </c>
       <c r="BE59" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="60" spans="1:57">
@@ -11289,7 +11289,7 @@
         <v>605</v>
       </c>
       <c r="BE60" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="61" spans="1:57">
@@ -11450,7 +11450,7 @@
         <v>605</v>
       </c>
       <c r="BE61" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="62" spans="1:57">
@@ -11611,7 +11611,7 @@
         <v>605</v>
       </c>
       <c r="BE62" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="63" spans="1:57">
@@ -11754,7 +11754,7 @@
         <v>605</v>
       </c>
       <c r="BE63" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="64" spans="1:57">
@@ -11900,7 +11900,7 @@
         <v>605</v>
       </c>
       <c r="BE64" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="65" spans="1:57">
@@ -12046,7 +12046,7 @@
         <v>605</v>
       </c>
       <c r="BE65" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="66" spans="1:57">
@@ -12198,7 +12198,7 @@
         <v>605</v>
       </c>
       <c r="BE66" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="67" spans="1:57">
@@ -12359,7 +12359,7 @@
         <v>605</v>
       </c>
       <c r="BE67" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="68" spans="1:57">
@@ -12520,7 +12520,7 @@
         <v>605</v>
       </c>
       <c r="BE68" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="69" spans="1:57">
@@ -12681,7 +12681,7 @@
         <v>605</v>
       </c>
       <c r="BE69" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="70" spans="1:57">
@@ -12842,7 +12842,7 @@
         <v>605</v>
       </c>
       <c r="BE70" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="71" spans="1:57">
@@ -13003,7 +13003,7 @@
         <v>605</v>
       </c>
       <c r="BE71" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="72" spans="1:57">
@@ -13149,7 +13149,7 @@
         <v>605</v>
       </c>
       <c r="BE72" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="73" spans="1:57">
@@ -13298,7 +13298,7 @@
         <v>605</v>
       </c>
       <c r="BE73" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="74" spans="1:57">
@@ -13444,7 +13444,7 @@
         <v>605</v>
       </c>
       <c r="BE74" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="75" spans="1:57">
@@ -13599,7 +13599,7 @@
         <v>605</v>
       </c>
       <c r="BE75" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="76" spans="1:57">
@@ -13754,7 +13754,7 @@
         <v>605</v>
       </c>
       <c r="BE76" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="77" spans="1:57">
@@ -13912,7 +13912,7 @@
         <v>605</v>
       </c>
       <c r="BE77" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="78" spans="1:57">
@@ -14073,7 +14073,7 @@
         <v>605</v>
       </c>
       <c r="BE78" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="79" spans="1:57">
@@ -14234,7 +14234,7 @@
         <v>605</v>
       </c>
       <c r="BE79" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="80" spans="1:57">
@@ -14395,7 +14395,7 @@
         <v>605</v>
       </c>
       <c r="BE80" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="81" spans="1:57">
@@ -14556,7 +14556,7 @@
         <v>605</v>
       </c>
       <c r="BE81" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="82" spans="1:57">
@@ -14717,7 +14717,7 @@
         <v>605</v>
       </c>
       <c r="BE82" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="83" spans="1:57">
@@ -14860,7 +14860,7 @@
         <v>605</v>
       </c>
       <c r="BE83" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="84" spans="1:57">
@@ -15021,7 +15021,7 @@
         <v>605</v>
       </c>
       <c r="BE84" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="85" spans="1:57">
@@ -15164,7 +15164,7 @@
         <v>605</v>
       </c>
       <c r="BE85" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="86" spans="1:57">
@@ -15316,7 +15316,7 @@
         <v>605</v>
       </c>
       <c r="BE86" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="87" spans="1:57">
@@ -15459,7 +15459,7 @@
         <v>605</v>
       </c>
       <c r="BE87" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="88" spans="1:57">
@@ -15602,7 +15602,7 @@
         <v>605</v>
       </c>
       <c r="BE88" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="89" spans="1:57">
@@ -15748,7 +15748,7 @@
         <v>605</v>
       </c>
       <c r="BE89" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="90" spans="1:57">
@@ -15915,7 +15915,7 @@
         <v>605</v>
       </c>
       <c r="BE90" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="91" spans="1:57">
@@ -16061,7 +16061,7 @@
         <v>605</v>
       </c>
       <c r="BE91" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="92" spans="1:57">
@@ -16222,7 +16222,7 @@
         <v>605</v>
       </c>
       <c r="BE92" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="93" spans="1:57">
@@ -16365,7 +16365,7 @@
         <v>605</v>
       </c>
       <c r="BE93" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="94" spans="1:57">
@@ -16511,7 +16511,7 @@
         <v>605</v>
       </c>
       <c r="BE94" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="95" spans="1:57">
@@ -16657,7 +16657,7 @@
         <v>605</v>
       </c>
       <c r="BE95" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="96" spans="1:57">
@@ -16800,7 +16800,7 @@
         <v>605</v>
       </c>
       <c r="BE96" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="97" spans="1:57">
@@ -16943,7 +16943,7 @@
         <v>605</v>
       </c>
       <c r="BE97" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="98" spans="1:57">
@@ -17086,7 +17086,7 @@
         <v>605</v>
       </c>
       <c r="BE98" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="99" spans="1:57">
@@ -17232,7 +17232,7 @@
         <v>605</v>
       </c>
       <c r="BE99" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="100" spans="1:57">
@@ -17384,7 +17384,7 @@
         <v>605</v>
       </c>
       <c r="BE100" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="101" spans="1:57">
@@ -17527,7 +17527,7 @@
         <v>605</v>
       </c>
       <c r="BE101" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="102" spans="1:57">
@@ -17670,7 +17670,7 @@
         <v>605</v>
       </c>
       <c r="BE102" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="103" spans="1:57">
@@ -17834,7 +17834,7 @@
         <v>605</v>
       </c>
       <c r="BE103" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="104" spans="1:57">
@@ -17977,7 +17977,7 @@
         <v>605</v>
       </c>
       <c r="BE104" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="105" spans="1:57">
@@ -18120,7 +18120,7 @@
         <v>605</v>
       </c>
       <c r="BE105" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="106" spans="1:57">
@@ -18281,7 +18281,7 @@
         <v>605</v>
       </c>
       <c r="BE106" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="107" spans="1:57">
@@ -18442,7 +18442,7 @@
         <v>605</v>
       </c>
       <c r="BE107" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="108" spans="1:57">
@@ -18603,7 +18603,7 @@
         <v>605</v>
       </c>
       <c r="BE108" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="109" spans="1:57">
@@ -18764,7 +18764,7 @@
         <v>605</v>
       </c>
       <c r="BE109" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="110" spans="1:57">
@@ -18925,7 +18925,7 @@
         <v>605</v>
       </c>
       <c r="BE110" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="111" spans="1:57">
@@ -19074,7 +19074,7 @@
         <v>605</v>
       </c>
       <c r="BE111" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="112" spans="1:57">
@@ -19217,7 +19217,7 @@
         <v>605</v>
       </c>
       <c r="BE112" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="113" spans="1:57">
@@ -19381,7 +19381,7 @@
         <v>605</v>
       </c>
       <c r="BE113" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="114" spans="1:57">
@@ -19524,7 +19524,7 @@
         <v>605</v>
       </c>
       <c r="BE114" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="115" spans="1:57">
@@ -19670,7 +19670,7 @@
         <v>605</v>
       </c>
       <c r="BE115" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="116" spans="1:57">
@@ -19813,7 +19813,7 @@
         <v>605</v>
       </c>
       <c r="BE116" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="117" spans="1:57">
@@ -19956,7 +19956,7 @@
         <v>605</v>
       </c>
       <c r="BE117" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="118" spans="1:57">
@@ -20102,7 +20102,7 @@
         <v>605</v>
       </c>
       <c r="BE118" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="119" spans="1:57">
@@ -20263,7 +20263,7 @@
         <v>605</v>
       </c>
       <c r="BE119" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="120" spans="1:57">
@@ -20412,7 +20412,7 @@
         <v>605</v>
       </c>
       <c r="BE120" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="121" spans="1:57">
@@ -20561,7 +20561,7 @@
         <v>605</v>
       </c>
       <c r="BE121" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="122" spans="1:57">
@@ -20704,7 +20704,7 @@
         <v>605</v>
       </c>
       <c r="BE122" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="123" spans="1:57">
@@ -20847,7 +20847,7 @@
         <v>605</v>
       </c>
       <c r="BE123" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="124" spans="1:57">
@@ -20993,7 +20993,7 @@
         <v>605</v>
       </c>
       <c r="BE124" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="125" spans="1:57">
@@ -21154,7 +21154,7 @@
         <v>605</v>
       </c>
       <c r="BE125" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="126" spans="1:57">
@@ -21315,7 +21315,7 @@
         <v>605</v>
       </c>
       <c r="BE126" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="127" spans="1:57">
@@ -21476,7 +21476,7 @@
         <v>605</v>
       </c>
       <c r="BE127" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="128" spans="1:57">
@@ -21619,7 +21619,7 @@
         <v>605</v>
       </c>
       <c r="BE128" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="129" spans="1:57">
@@ -21780,7 +21780,7 @@
         <v>605</v>
       </c>
       <c r="BE129" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="130" spans="1:57">
@@ -21929,7 +21929,7 @@
         <v>605</v>
       </c>
       <c r="BE130" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="131" spans="1:57">
@@ -22072,7 +22072,7 @@
         <v>605</v>
       </c>
       <c r="BE131" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="132" spans="1:57">
@@ -22215,7 +22215,7 @@
         <v>605</v>
       </c>
       <c r="BE132" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="133" spans="1:57">
@@ -22358,7 +22358,7 @@
         <v>605</v>
       </c>
       <c r="BE133" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="134" spans="1:57">
@@ -22501,7 +22501,7 @@
         <v>605</v>
       </c>
       <c r="BE134" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="135" spans="1:57">
@@ -22644,7 +22644,7 @@
         <v>605</v>
       </c>
       <c r="BE135" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="136" spans="1:57">
@@ -22787,7 +22787,7 @@
         <v>605</v>
       </c>
       <c r="BE136" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="137" spans="1:57">
@@ -22933,7 +22933,7 @@
         <v>605</v>
       </c>
       <c r="BE137" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="138" spans="1:57">
@@ -23100,7 +23100,7 @@
         <v>605</v>
       </c>
       <c r="BE138" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="139" spans="1:57">
@@ -23243,7 +23243,7 @@
         <v>605</v>
       </c>
       <c r="BE139" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="140" spans="1:57">
@@ -23386,7 +23386,7 @@
         <v>605</v>
       </c>
       <c r="BE140" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="141" spans="1:57">
@@ -23550,7 +23550,7 @@
         <v>605</v>
       </c>
       <c r="BE141" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="142" spans="1:57">
@@ -23693,7 +23693,7 @@
         <v>605</v>
       </c>
       <c r="BE142" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="143" spans="1:57">
@@ -23854,7 +23854,7 @@
         <v>605</v>
       </c>
       <c r="BE143" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="144" spans="1:57">
@@ -23997,7 +23997,7 @@
         <v>605</v>
       </c>
       <c r="BE144" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="145" spans="1:57">
@@ -24140,7 +24140,7 @@
         <v>605</v>
       </c>
       <c r="BE145" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="146" spans="1:57">
@@ -24292,7 +24292,7 @@
         <v>605</v>
       </c>
       <c r="BE146" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="147" spans="1:57">
@@ -24438,7 +24438,7 @@
         <v>605</v>
       </c>
       <c r="BE147" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="148" spans="1:57">
@@ -24584,7 +24584,7 @@
         <v>605</v>
       </c>
       <c r="BE148" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="149" spans="1:57">
@@ -24727,7 +24727,7 @@
         <v>605</v>
       </c>
       <c r="BE149" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="150" spans="1:57">
@@ -24876,7 +24876,7 @@
         <v>605</v>
       </c>
       <c r="BE150" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="151" spans="1:57">
@@ -25022,7 +25022,7 @@
         <v>605</v>
       </c>
       <c r="BE151" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="152" spans="1:57">
@@ -25165,7 +25165,7 @@
         <v>605</v>
       </c>
       <c r="BE152" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="153" spans="1:57">
@@ -25308,7 +25308,7 @@
         <v>605</v>
       </c>
       <c r="BE153" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="154" spans="1:57">
@@ -25469,7 +25469,7 @@
         <v>605</v>
       </c>
       <c r="BE154" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="155" spans="1:57">
@@ -25630,7 +25630,7 @@
         <v>605</v>
       </c>
       <c r="BE155" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="156" spans="1:57">
@@ -25791,7 +25791,7 @@
         <v>605</v>
       </c>
       <c r="BE156" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="157" spans="1:57">
@@ -25952,7 +25952,7 @@
         <v>605</v>
       </c>
       <c r="BE157" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="158" spans="1:57">
@@ -26098,7 +26098,7 @@
         <v>605</v>
       </c>
       <c r="BE158" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="159" spans="1:57">
@@ -26241,7 +26241,7 @@
         <v>605</v>
       </c>
       <c r="BE159" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="160" spans="1:57">
@@ -26393,7 +26393,7 @@
         <v>605</v>
       </c>
       <c r="BE160" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="161" spans="1:57">
@@ -26554,7 +26554,7 @@
         <v>605</v>
       </c>
       <c r="BE161" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="162" spans="1:57">
@@ -26697,7 +26697,7 @@
         <v>605</v>
       </c>
       <c r="BE162" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="163" spans="1:57">
@@ -26846,7 +26846,7 @@
         <v>605</v>
       </c>
       <c r="BE163" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="164" spans="1:57">
@@ -26989,7 +26989,7 @@
         <v>605</v>
       </c>
       <c r="BE164" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="165" spans="1:57">
@@ -27150,7 +27150,7 @@
         <v>605</v>
       </c>
       <c r="BE165" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="166" spans="1:57">
@@ -27296,7 +27296,7 @@
         <v>605</v>
       </c>
       <c r="BE166" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="167" spans="1:57">
@@ -27439,7 +27439,7 @@
         <v>605</v>
       </c>
       <c r="BE167" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="168" spans="1:57">
@@ -27603,7 +27603,7 @@
         <v>605</v>
       </c>
       <c r="BE168" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="169" spans="1:57">
@@ -27749,7 +27749,7 @@
         <v>605</v>
       </c>
       <c r="BE169" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="170" spans="1:57">
@@ -27901,7 +27901,7 @@
         <v>605</v>
       </c>
       <c r="BE170" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="171" spans="1:57">
@@ -28053,7 +28053,7 @@
         <v>605</v>
       </c>
       <c r="BE171" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="172" spans="1:57">
@@ -28214,7 +28214,7 @@
         <v>605</v>
       </c>
       <c r="BE172" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="173" spans="1:57">
@@ -28378,7 +28378,7 @@
         <v>605</v>
       </c>
       <c r="BE173" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="174" spans="1:57">
@@ -28539,7 +28539,7 @@
         <v>605</v>
       </c>
       <c r="BE174" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="175" spans="1:57">
@@ -28691,7 +28691,7 @@
         <v>605</v>
       </c>
       <c r="BE175" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="176" spans="1:57">
@@ -28834,7 +28834,7 @@
         <v>605</v>
       </c>
       <c r="BE176" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="177" spans="1:57">
@@ -28977,7 +28977,7 @@
         <v>605</v>
       </c>
       <c r="BE177" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="178" spans="1:57">
@@ -29138,7 +29138,7 @@
         <v>605</v>
       </c>
       <c r="BE178" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="179" spans="1:57">
@@ -29281,7 +29281,7 @@
         <v>605</v>
       </c>
       <c r="BE179" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="180" spans="1:57">
@@ -29424,7 +29424,7 @@
         <v>605</v>
       </c>
       <c r="BE180" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="181" spans="1:57">
@@ -29567,7 +29567,7 @@
         <v>605</v>
       </c>
       <c r="BE181" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="182" spans="1:57">
@@ -29710,7 +29710,7 @@
         <v>605</v>
       </c>
       <c r="BE182" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
     <row r="183" spans="1:57">
@@ -29871,7 +29871,7 @@
         <v>605</v>
       </c>
       <c r="BE183" s="2">
-        <v>46044.29181770714</v>
+        <v>46044.8802823589</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily dashboard refresh 2026-01-22 21:17
</commit_message>
<xml_diff>
--- a/data/Fail.xlsx
+++ b/data/Fail.xlsx
@@ -2536,7 +2536,7 @@
         <v>605</v>
       </c>
       <c r="BE2" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="3" spans="1:57">
@@ -2679,7 +2679,7 @@
         <v>605</v>
       </c>
       <c r="BE3" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="4" spans="1:57">
@@ -2840,7 +2840,7 @@
         <v>605</v>
       </c>
       <c r="BE4" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="5" spans="1:57">
@@ -3004,7 +3004,7 @@
         <v>605</v>
       </c>
       <c r="BE5" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="6" spans="1:57">
@@ -3165,7 +3165,7 @@
         <v>605</v>
       </c>
       <c r="BE6" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="7" spans="1:57">
@@ -3320,7 +3320,7 @@
         <v>605</v>
       </c>
       <c r="BE7" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="8" spans="1:57">
@@ -3481,7 +3481,7 @@
         <v>605</v>
       </c>
       <c r="BE8" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="9" spans="1:57">
@@ -3624,7 +3624,7 @@
         <v>605</v>
       </c>
       <c r="BE9" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="10" spans="1:57">
@@ -3767,7 +3767,7 @@
         <v>605</v>
       </c>
       <c r="BE10" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="11" spans="1:57">
@@ -3913,7 +3913,7 @@
         <v>605</v>
       </c>
       <c r="BE11" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="12" spans="1:57">
@@ -4074,7 +4074,7 @@
         <v>605</v>
       </c>
       <c r="BE12" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="13" spans="1:57">
@@ -4235,7 +4235,7 @@
         <v>605</v>
       </c>
       <c r="BE13" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="14" spans="1:57">
@@ -4396,7 +4396,7 @@
         <v>605</v>
       </c>
       <c r="BE14" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="15" spans="1:57">
@@ -4545,7 +4545,7 @@
         <v>605</v>
       </c>
       <c r="BE15" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="16" spans="1:57">
@@ -4706,7 +4706,7 @@
         <v>605</v>
       </c>
       <c r="BE16" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="17" spans="1:57">
@@ -4852,7 +4852,7 @@
         <v>605</v>
       </c>
       <c r="BE17" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="18" spans="1:57">
@@ -4995,7 +4995,7 @@
         <v>605</v>
       </c>
       <c r="BE18" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="19" spans="1:57">
@@ -5156,7 +5156,7 @@
         <v>605</v>
       </c>
       <c r="BE19" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="20" spans="1:57">
@@ -5317,7 +5317,7 @@
         <v>605</v>
       </c>
       <c r="BE20" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="21" spans="1:57">
@@ -5478,7 +5478,7 @@
         <v>605</v>
       </c>
       <c r="BE21" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="22" spans="1:57">
@@ -5630,7 +5630,7 @@
         <v>605</v>
       </c>
       <c r="BE22" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="23" spans="1:57">
@@ -5776,7 +5776,7 @@
         <v>605</v>
       </c>
       <c r="BE23" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="24" spans="1:57">
@@ -5937,7 +5937,7 @@
         <v>605</v>
       </c>
       <c r="BE24" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="25" spans="1:57">
@@ -6080,7 +6080,7 @@
         <v>605</v>
       </c>
       <c r="BE25" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="26" spans="1:57">
@@ -6241,7 +6241,7 @@
         <v>605</v>
       </c>
       <c r="BE26" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="27" spans="1:57">
@@ -6384,7 +6384,7 @@
         <v>605</v>
       </c>
       <c r="BE27" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="28" spans="1:57">
@@ -6527,7 +6527,7 @@
         <v>605</v>
       </c>
       <c r="BE28" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="29" spans="1:57">
@@ -6670,7 +6670,7 @@
         <v>605</v>
       </c>
       <c r="BE29" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="30" spans="1:57">
@@ -6813,7 +6813,7 @@
         <v>605</v>
       </c>
       <c r="BE30" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="31" spans="1:57">
@@ -6974,7 +6974,7 @@
         <v>605</v>
       </c>
       <c r="BE31" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="32" spans="1:57">
@@ -7120,7 +7120,7 @@
         <v>605</v>
       </c>
       <c r="BE32" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="33" spans="1:57">
@@ -7266,7 +7266,7 @@
         <v>605</v>
       </c>
       <c r="BE33" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="34" spans="1:57">
@@ -7418,7 +7418,7 @@
         <v>605</v>
       </c>
       <c r="BE34" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="35" spans="1:57">
@@ -7564,7 +7564,7 @@
         <v>605</v>
       </c>
       <c r="BE35" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="36" spans="1:57">
@@ -7716,7 +7716,7 @@
         <v>605</v>
       </c>
       <c r="BE36" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="37" spans="1:57">
@@ -7859,7 +7859,7 @@
         <v>605</v>
       </c>
       <c r="BE37" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="38" spans="1:57">
@@ -8002,7 +8002,7 @@
         <v>605</v>
       </c>
       <c r="BE38" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="39" spans="1:57">
@@ -8163,7 +8163,7 @@
         <v>605</v>
       </c>
       <c r="BE39" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="40" spans="1:57">
@@ -8306,7 +8306,7 @@
         <v>605</v>
       </c>
       <c r="BE40" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="41" spans="1:57">
@@ -8452,7 +8452,7 @@
         <v>605</v>
       </c>
       <c r="BE41" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="42" spans="1:57">
@@ -8604,7 +8604,7 @@
         <v>605</v>
       </c>
       <c r="BE42" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="43" spans="1:57">
@@ -8747,7 +8747,7 @@
         <v>605</v>
       </c>
       <c r="BE43" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="44" spans="1:57">
@@ -8908,7 +8908,7 @@
         <v>605</v>
       </c>
       <c r="BE44" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="45" spans="1:57">
@@ -9054,7 +9054,7 @@
         <v>605</v>
       </c>
       <c r="BE45" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="46" spans="1:57">
@@ -9209,7 +9209,7 @@
         <v>605</v>
       </c>
       <c r="BE46" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="47" spans="1:57">
@@ -9352,7 +9352,7 @@
         <v>605</v>
       </c>
       <c r="BE47" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="48" spans="1:57">
@@ -9513,7 +9513,7 @@
         <v>605</v>
       </c>
       <c r="BE48" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="49" spans="1:57">
@@ -9656,7 +9656,7 @@
         <v>605</v>
       </c>
       <c r="BE49" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="50" spans="1:57">
@@ -9808,7 +9808,7 @@
         <v>605</v>
       </c>
       <c r="BE50" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="51" spans="1:57">
@@ -9960,7 +9960,7 @@
         <v>605</v>
       </c>
       <c r="BE51" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="52" spans="1:57">
@@ -10109,7 +10109,7 @@
         <v>605</v>
       </c>
       <c r="BE52" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="53" spans="1:57">
@@ -10252,7 +10252,7 @@
         <v>605</v>
       </c>
       <c r="BE53" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="54" spans="1:57">
@@ -10395,7 +10395,7 @@
         <v>605</v>
       </c>
       <c r="BE54" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="55" spans="1:57">
@@ -10538,7 +10538,7 @@
         <v>605</v>
       </c>
       <c r="BE55" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="56" spans="1:57">
@@ -10690,7 +10690,7 @@
         <v>605</v>
       </c>
       <c r="BE56" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="57" spans="1:57">
@@ -10842,7 +10842,7 @@
         <v>605</v>
       </c>
       <c r="BE57" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="58" spans="1:57">
@@ -11003,7 +11003,7 @@
         <v>605</v>
       </c>
       <c r="BE58" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="59" spans="1:57">
@@ -11146,7 +11146,7 @@
         <v>605</v>
       </c>
       <c r="BE59" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="60" spans="1:57">
@@ -11289,7 +11289,7 @@
         <v>605</v>
       </c>
       <c r="BE60" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="61" spans="1:57">
@@ -11450,7 +11450,7 @@
         <v>605</v>
       </c>
       <c r="BE61" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="62" spans="1:57">
@@ -11611,7 +11611,7 @@
         <v>605</v>
       </c>
       <c r="BE62" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="63" spans="1:57">
@@ -11754,7 +11754,7 @@
         <v>605</v>
       </c>
       <c r="BE63" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="64" spans="1:57">
@@ -11900,7 +11900,7 @@
         <v>605</v>
       </c>
       <c r="BE64" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="65" spans="1:57">
@@ -12046,7 +12046,7 @@
         <v>605</v>
       </c>
       <c r="BE65" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="66" spans="1:57">
@@ -12198,7 +12198,7 @@
         <v>605</v>
       </c>
       <c r="BE66" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="67" spans="1:57">
@@ -12359,7 +12359,7 @@
         <v>605</v>
       </c>
       <c r="BE67" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="68" spans="1:57">
@@ -12520,7 +12520,7 @@
         <v>605</v>
       </c>
       <c r="BE68" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="69" spans="1:57">
@@ -12681,7 +12681,7 @@
         <v>605</v>
       </c>
       <c r="BE69" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="70" spans="1:57">
@@ -12842,7 +12842,7 @@
         <v>605</v>
       </c>
       <c r="BE70" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="71" spans="1:57">
@@ -13003,7 +13003,7 @@
         <v>605</v>
       </c>
       <c r="BE71" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="72" spans="1:57">
@@ -13149,7 +13149,7 @@
         <v>605</v>
       </c>
       <c r="BE72" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="73" spans="1:57">
@@ -13298,7 +13298,7 @@
         <v>605</v>
       </c>
       <c r="BE73" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="74" spans="1:57">
@@ -13444,7 +13444,7 @@
         <v>605</v>
       </c>
       <c r="BE74" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="75" spans="1:57">
@@ -13599,7 +13599,7 @@
         <v>605</v>
       </c>
       <c r="BE75" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="76" spans="1:57">
@@ -13754,7 +13754,7 @@
         <v>605</v>
       </c>
       <c r="BE76" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="77" spans="1:57">
@@ -13912,7 +13912,7 @@
         <v>605</v>
       </c>
       <c r="BE77" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="78" spans="1:57">
@@ -14073,7 +14073,7 @@
         <v>605</v>
       </c>
       <c r="BE78" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="79" spans="1:57">
@@ -14234,7 +14234,7 @@
         <v>605</v>
       </c>
       <c r="BE79" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="80" spans="1:57">
@@ -14395,7 +14395,7 @@
         <v>605</v>
       </c>
       <c r="BE80" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="81" spans="1:57">
@@ -14556,7 +14556,7 @@
         <v>605</v>
       </c>
       <c r="BE81" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="82" spans="1:57">
@@ -14717,7 +14717,7 @@
         <v>605</v>
       </c>
       <c r="BE82" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="83" spans="1:57">
@@ -14860,7 +14860,7 @@
         <v>605</v>
       </c>
       <c r="BE83" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="84" spans="1:57">
@@ -15021,7 +15021,7 @@
         <v>605</v>
       </c>
       <c r="BE84" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="85" spans="1:57">
@@ -15164,7 +15164,7 @@
         <v>605</v>
       </c>
       <c r="BE85" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="86" spans="1:57">
@@ -15316,7 +15316,7 @@
         <v>605</v>
       </c>
       <c r="BE86" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="87" spans="1:57">
@@ -15459,7 +15459,7 @@
         <v>605</v>
       </c>
       <c r="BE87" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="88" spans="1:57">
@@ -15602,7 +15602,7 @@
         <v>605</v>
       </c>
       <c r="BE88" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="89" spans="1:57">
@@ -15748,7 +15748,7 @@
         <v>605</v>
       </c>
       <c r="BE89" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="90" spans="1:57">
@@ -15915,7 +15915,7 @@
         <v>605</v>
       </c>
       <c r="BE90" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="91" spans="1:57">
@@ -16061,7 +16061,7 @@
         <v>605</v>
       </c>
       <c r="BE91" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="92" spans="1:57">
@@ -16222,7 +16222,7 @@
         <v>605</v>
       </c>
       <c r="BE92" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="93" spans="1:57">
@@ -16365,7 +16365,7 @@
         <v>605</v>
       </c>
       <c r="BE93" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="94" spans="1:57">
@@ -16511,7 +16511,7 @@
         <v>605</v>
       </c>
       <c r="BE94" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="95" spans="1:57">
@@ -16657,7 +16657,7 @@
         <v>605</v>
       </c>
       <c r="BE95" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="96" spans="1:57">
@@ -16800,7 +16800,7 @@
         <v>605</v>
       </c>
       <c r="BE96" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="97" spans="1:57">
@@ -16943,7 +16943,7 @@
         <v>605</v>
       </c>
       <c r="BE97" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="98" spans="1:57">
@@ -17086,7 +17086,7 @@
         <v>605</v>
       </c>
       <c r="BE98" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="99" spans="1:57">
@@ -17232,7 +17232,7 @@
         <v>605</v>
       </c>
       <c r="BE99" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="100" spans="1:57">
@@ -17384,7 +17384,7 @@
         <v>605</v>
       </c>
       <c r="BE100" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="101" spans="1:57">
@@ -17527,7 +17527,7 @@
         <v>605</v>
       </c>
       <c r="BE101" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="102" spans="1:57">
@@ -17670,7 +17670,7 @@
         <v>605</v>
       </c>
       <c r="BE102" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="103" spans="1:57">
@@ -17834,7 +17834,7 @@
         <v>605</v>
       </c>
       <c r="BE103" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="104" spans="1:57">
@@ -17977,7 +17977,7 @@
         <v>605</v>
       </c>
       <c r="BE104" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="105" spans="1:57">
@@ -18120,7 +18120,7 @@
         <v>605</v>
       </c>
       <c r="BE105" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="106" spans="1:57">
@@ -18281,7 +18281,7 @@
         <v>605</v>
       </c>
       <c r="BE106" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="107" spans="1:57">
@@ -18442,7 +18442,7 @@
         <v>605</v>
       </c>
       <c r="BE107" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="108" spans="1:57">
@@ -18603,7 +18603,7 @@
         <v>605</v>
       </c>
       <c r="BE108" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="109" spans="1:57">
@@ -18764,7 +18764,7 @@
         <v>605</v>
       </c>
       <c r="BE109" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="110" spans="1:57">
@@ -18925,7 +18925,7 @@
         <v>605</v>
       </c>
       <c r="BE110" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="111" spans="1:57">
@@ -19074,7 +19074,7 @@
         <v>605</v>
       </c>
       <c r="BE111" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="112" spans="1:57">
@@ -19217,7 +19217,7 @@
         <v>605</v>
       </c>
       <c r="BE112" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="113" spans="1:57">
@@ -19381,7 +19381,7 @@
         <v>605</v>
       </c>
       <c r="BE113" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="114" spans="1:57">
@@ -19524,7 +19524,7 @@
         <v>605</v>
       </c>
       <c r="BE114" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="115" spans="1:57">
@@ -19670,7 +19670,7 @@
         <v>605</v>
       </c>
       <c r="BE115" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="116" spans="1:57">
@@ -19813,7 +19813,7 @@
         <v>605</v>
       </c>
       <c r="BE116" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="117" spans="1:57">
@@ -19956,7 +19956,7 @@
         <v>605</v>
       </c>
       <c r="BE117" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="118" spans="1:57">
@@ -20102,7 +20102,7 @@
         <v>605</v>
       </c>
       <c r="BE118" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="119" spans="1:57">
@@ -20263,7 +20263,7 @@
         <v>605</v>
       </c>
       <c r="BE119" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="120" spans="1:57">
@@ -20412,7 +20412,7 @@
         <v>605</v>
       </c>
       <c r="BE120" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="121" spans="1:57">
@@ -20561,7 +20561,7 @@
         <v>605</v>
       </c>
       <c r="BE121" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="122" spans="1:57">
@@ -20704,7 +20704,7 @@
         <v>605</v>
       </c>
       <c r="BE122" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="123" spans="1:57">
@@ -20847,7 +20847,7 @@
         <v>605</v>
       </c>
       <c r="BE123" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="124" spans="1:57">
@@ -20993,7 +20993,7 @@
         <v>605</v>
       </c>
       <c r="BE124" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="125" spans="1:57">
@@ -21154,7 +21154,7 @@
         <v>605</v>
       </c>
       <c r="BE125" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="126" spans="1:57">
@@ -21315,7 +21315,7 @@
         <v>605</v>
       </c>
       <c r="BE126" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="127" spans="1:57">
@@ -21476,7 +21476,7 @@
         <v>605</v>
       </c>
       <c r="BE127" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="128" spans="1:57">
@@ -21619,7 +21619,7 @@
         <v>605</v>
       </c>
       <c r="BE128" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="129" spans="1:57">
@@ -21780,7 +21780,7 @@
         <v>605</v>
       </c>
       <c r="BE129" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="130" spans="1:57">
@@ -21929,7 +21929,7 @@
         <v>605</v>
       </c>
       <c r="BE130" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="131" spans="1:57">
@@ -22072,7 +22072,7 @@
         <v>605</v>
       </c>
       <c r="BE131" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="132" spans="1:57">
@@ -22215,7 +22215,7 @@
         <v>605</v>
       </c>
       <c r="BE132" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="133" spans="1:57">
@@ -22358,7 +22358,7 @@
         <v>605</v>
       </c>
       <c r="BE133" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="134" spans="1:57">
@@ -22501,7 +22501,7 @@
         <v>605</v>
       </c>
       <c r="BE134" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="135" spans="1:57">
@@ -22644,7 +22644,7 @@
         <v>605</v>
       </c>
       <c r="BE135" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="136" spans="1:57">
@@ -22787,7 +22787,7 @@
         <v>605</v>
       </c>
       <c r="BE136" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="137" spans="1:57">
@@ -22933,7 +22933,7 @@
         <v>605</v>
       </c>
       <c r="BE137" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="138" spans="1:57">
@@ -23100,7 +23100,7 @@
         <v>605</v>
       </c>
       <c r="BE138" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="139" spans="1:57">
@@ -23243,7 +23243,7 @@
         <v>605</v>
       </c>
       <c r="BE139" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="140" spans="1:57">
@@ -23386,7 +23386,7 @@
         <v>605</v>
       </c>
       <c r="BE140" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="141" spans="1:57">
@@ -23550,7 +23550,7 @@
         <v>605</v>
       </c>
       <c r="BE141" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="142" spans="1:57">
@@ -23693,7 +23693,7 @@
         <v>605</v>
       </c>
       <c r="BE142" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="143" spans="1:57">
@@ -23854,7 +23854,7 @@
         <v>605</v>
       </c>
       <c r="BE143" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="144" spans="1:57">
@@ -23997,7 +23997,7 @@
         <v>605</v>
       </c>
       <c r="BE144" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="145" spans="1:57">
@@ -24140,7 +24140,7 @@
         <v>605</v>
       </c>
       <c r="BE145" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="146" spans="1:57">
@@ -24292,7 +24292,7 @@
         <v>605</v>
       </c>
       <c r="BE146" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="147" spans="1:57">
@@ -24438,7 +24438,7 @@
         <v>605</v>
       </c>
       <c r="BE147" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="148" spans="1:57">
@@ -24584,7 +24584,7 @@
         <v>605</v>
       </c>
       <c r="BE148" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="149" spans="1:57">
@@ -24727,7 +24727,7 @@
         <v>605</v>
       </c>
       <c r="BE149" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="150" spans="1:57">
@@ -24876,7 +24876,7 @@
         <v>605</v>
       </c>
       <c r="BE150" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="151" spans="1:57">
@@ -25022,7 +25022,7 @@
         <v>605</v>
       </c>
       <c r="BE151" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="152" spans="1:57">
@@ -25165,7 +25165,7 @@
         <v>605</v>
       </c>
       <c r="BE152" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="153" spans="1:57">
@@ -25308,7 +25308,7 @@
         <v>605</v>
       </c>
       <c r="BE153" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="154" spans="1:57">
@@ -25469,7 +25469,7 @@
         <v>605</v>
       </c>
       <c r="BE154" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="155" spans="1:57">
@@ -25630,7 +25630,7 @@
         <v>605</v>
       </c>
       <c r="BE155" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="156" spans="1:57">
@@ -25791,7 +25791,7 @@
         <v>605</v>
       </c>
       <c r="BE156" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="157" spans="1:57">
@@ -25952,7 +25952,7 @@
         <v>605</v>
       </c>
       <c r="BE157" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="158" spans="1:57">
@@ -26098,7 +26098,7 @@
         <v>605</v>
       </c>
       <c r="BE158" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="159" spans="1:57">
@@ -26241,7 +26241,7 @@
         <v>605</v>
       </c>
       <c r="BE159" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="160" spans="1:57">
@@ -26393,7 +26393,7 @@
         <v>605</v>
       </c>
       <c r="BE160" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="161" spans="1:57">
@@ -26554,7 +26554,7 @@
         <v>605</v>
       </c>
       <c r="BE161" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="162" spans="1:57">
@@ -26697,7 +26697,7 @@
         <v>605</v>
       </c>
       <c r="BE162" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="163" spans="1:57">
@@ -26846,7 +26846,7 @@
         <v>605</v>
       </c>
       <c r="BE163" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="164" spans="1:57">
@@ -26989,7 +26989,7 @@
         <v>605</v>
       </c>
       <c r="BE164" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="165" spans="1:57">
@@ -27150,7 +27150,7 @@
         <v>605</v>
       </c>
       <c r="BE165" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="166" spans="1:57">
@@ -27296,7 +27296,7 @@
         <v>605</v>
       </c>
       <c r="BE166" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="167" spans="1:57">
@@ -27439,7 +27439,7 @@
         <v>605</v>
       </c>
       <c r="BE167" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="168" spans="1:57">
@@ -27603,7 +27603,7 @@
         <v>605</v>
       </c>
       <c r="BE168" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="169" spans="1:57">
@@ -27749,7 +27749,7 @@
         <v>605</v>
       </c>
       <c r="BE169" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="170" spans="1:57">
@@ -27901,7 +27901,7 @@
         <v>605</v>
       </c>
       <c r="BE170" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="171" spans="1:57">
@@ -28053,7 +28053,7 @@
         <v>605</v>
       </c>
       <c r="BE171" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="172" spans="1:57">
@@ -28214,7 +28214,7 @@
         <v>605</v>
       </c>
       <c r="BE172" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="173" spans="1:57">
@@ -28378,7 +28378,7 @@
         <v>605</v>
       </c>
       <c r="BE173" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="174" spans="1:57">
@@ -28539,7 +28539,7 @@
         <v>605</v>
       </c>
       <c r="BE174" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="175" spans="1:57">
@@ -28691,7 +28691,7 @@
         <v>605</v>
       </c>
       <c r="BE175" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="176" spans="1:57">
@@ -28834,7 +28834,7 @@
         <v>605</v>
       </c>
       <c r="BE176" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="177" spans="1:57">
@@ -28977,7 +28977,7 @@
         <v>605</v>
       </c>
       <c r="BE177" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="178" spans="1:57">
@@ -29138,7 +29138,7 @@
         <v>605</v>
       </c>
       <c r="BE178" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="179" spans="1:57">
@@ -29281,7 +29281,7 @@
         <v>605</v>
       </c>
       <c r="BE179" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="180" spans="1:57">
@@ -29424,7 +29424,7 @@
         <v>605</v>
       </c>
       <c r="BE180" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="181" spans="1:57">
@@ -29567,7 +29567,7 @@
         <v>605</v>
       </c>
       <c r="BE181" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="182" spans="1:57">
@@ -29710,7 +29710,7 @@
         <v>605</v>
       </c>
       <c r="BE182" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
     <row r="183" spans="1:57">
@@ -29871,7 +29871,7 @@
         <v>605</v>
       </c>
       <c r="BE183" s="2">
-        <v>46044.8802823589</v>
+        <v>46044.88673615588</v>
       </c>
     </row>
   </sheetData>

</xml_diff>